<commit_message>
Spalte Von in der Excel und im Reset-Skript
</commit_message>
<xml_diff>
--- a/skills_daten.xlsx
+++ b/skills_daten.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,7 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -481,6 +482,11 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Tipp</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Von</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kopfzeilenformatierung und Filterbereich fuer Spalte Von nachziehen
G1 erhaelt dieselbe Formatierung (Fuellung, fett, zentriert) wie die
uebrigen Kopfzellen, und der AutoFilter deckt neu alle sieben Spalten
ab (A1:G101), damit Sortieren/Filtern die Von-Werte nicht von ihren
Zeilen trennt.
</commit_message>
<xml_diff>
--- a/skills_daten.xlsx
+++ b/skills_daten.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Kategorien" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$G$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stufen'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorien'!$A$1:$C$10</definedName>
   </definedNames>
@@ -484,7 +484,7 @@
           <t>Tipp</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Von</t>
         </is>
@@ -3691,7 +3691,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F101"/>
+  <autoFilter ref="A1:G101"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Stufe" error="Bitte Hoch, Mittel oder Tief wählen." promptTitle="Stufe" prompt="Hoch / Mittel / Tief" type="list">
       <formula1>"Hoch,Mittel,Tief"</formula1>

</xml_diff>

<commit_message>
Spalte Ergaenzt durch die Datenkette, Detail-Dialog nennt beide Beitragenden
</commit_message>
<xml_diff>
--- a/skills_daten.xlsx
+++ b/skills_daten.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Kategorien" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$H$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stufen'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorien'!$A$1:$C$10</definedName>
   </definedNames>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -451,6 +451,7 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -489,6 +490,11 @@
           <t>Von</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ergaenzt</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3691,7 +3697,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G101"/>
+  <autoFilter ref="A1:H101"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Stufe" error="Bitte Hoch, Mittel oder Tief wählen." promptTitle="Stufe" prompt="Hoch / Mittel / Tief" type="list">
       <formula1>"Hoch,Mittel,Tief"</formula1>

</xml_diff>

<commit_message>
Fix: Link1-Link3 im Blatt Skills ergaenzt, ANLEITUNG.md nachgezogen
skills_daten.xlsx hatte im Blatt Skills nur acht Spalten (bis Ergaenzt) -
die drei Link-Spalten fehlten, obwohl CLAUDE.md und ANLEITUNG.md sie als
vorhanden beschrieben. Wer von Hand eine Bezugsquelle eintragen wollte, fand
in Excel nichts.

Header Link1/Link2/Link3 ergaenzt (Spaltenbreite 40, wie in
tools/seed_excel.py), Autofilter auf A1:K101 erweitert. Verifiziert:
Kopfzeile hat die erwarteten elf Namen, das Stufe-Dropdown auf Spalte A
besteht weiter, 101 Zeilen unveraendert, Autofilter korrekt. `uv run build.py`
danach: docs/ bleibt unveraendert (git diff --stat docs/ ist leer) - der
Umbau hat keine erzeugten Inhalte beruehrt.

ANLEITUNG.md: die drei Link-Spalten in der Spaltentabelle ergaenzt, damit
sie nicht mehr im Widerspruch zum spaeteren Abschnitt "Bezugsquellen" steht.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills_daten.xlsx
+++ b/skills_daten.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Kategorien" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$H$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$K$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stufen'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorien'!$A$1:$C$10</definedName>
   </definedNames>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -452,6 +452,9 @@
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -495,6 +498,21 @@
           <t>Ergaenzt</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Link1</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Link2</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Link3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3697,7 +3715,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H101"/>
+  <autoFilter ref="A1:K101"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Stufe" error="Bitte Hoch, Mittel oder Tief wählen." promptTitle="Stufe" prompt="Hoch / Mittel / Tief" type="list">
       <formula1>"Hoch,Mittel,Tief"</formula1>

</xml_diff>